<commit_message>
add Updated files to upload React package to Nexus
</commit_message>
<xml_diff>
--- a/Inventroy.xlsx
+++ b/Inventroy.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VDR000691\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VDR000691\Documents\Tawn-Scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE8DAA0F-CBC5-42B7-8579-D710D2B4734F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C57FCEAA-5B50-4CB0-A6A7-0E1E2B0045C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{2952D06E-A856-41C4-A812-1B0185948966}"/>
   </bookViews>
@@ -513,13 +513,13 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF92D050"/>
+      <color rgb="FFC00000"/>
       <name val="Aptos Display"/>
       <family val="2"/>
       <scheme val="major"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -538,6 +538,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -552,7 +558,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
@@ -567,15 +573,12 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -583,63 +586,7 @@
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="14">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF0070C0"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF0070C0"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF0070C0"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF0070C0"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF0070C0"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF0070C0"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF0070C0"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="8">
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -676,6 +623,14 @@
         <scheme val="major"/>
       </font>
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF0070C0"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2946,22 +2901,23 @@
   <autoFilter ref="A1:J74" xr:uid="{332BA11F-8A65-4D33-BD80-8CAB66DCB57E}">
     <filterColumn colId="4">
       <filters>
-        <filter val="Java"/>
+        <filter val="React"/>
+        <filter val="React + TypeScript + Node.js"/>
       </filters>
     </filterColumn>
   </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J24">
-    <sortCondition sortBy="cellColor" ref="A2:A74" dxfId="1"/>
+    <sortCondition sortBy="cellColor" ref="A2:A74" dxfId="7"/>
   </sortState>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{3950FF09-387A-460E-9A47-9DDFFB93E0AC}" name="Job Name" dataDxfId="13" dataCellStyle="Hyperlink"/>
+    <tableColumn id="1" xr3:uid="{3950FF09-387A-460E-9A47-9DDFFB93E0AC}" name="Job Name" dataDxfId="6" dataCellStyle="Hyperlink"/>
     <tableColumn id="2" xr3:uid="{6F6F8DE8-D558-4364-9A59-13F5A6E112D7}" name="URL" dataCellStyle="Hyperlink"/>
-    <tableColumn id="3" xr3:uid="{04F312B6-748C-4380-9A58-005F09BCD38F}" name="Last Build" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{6BB0F30E-FA6E-40B9-88DC-F336A66A15EA}" name="LOB/Project" dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{7EEF8C9E-E28F-4C2F-82B3-CCDBBE2BAE5B}" name="Technology Stack" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{C76712CA-C3D0-400A-A5B0-1590E99A3801}" name="Framework" dataDxfId="12"/>
-    <tableColumn id="7" xr3:uid="{D40351DA-4625-4AED-92C1-8C733CE6AAF1}" name="Runtime" dataDxfId="10"/>
-    <tableColumn id="11" xr3:uid="{049BCF70-240C-47F6-81A7-D6DCBBA621E4}" name="Shared Library" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{04F312B6-748C-4380-9A58-005F09BCD38F}" name="Last Build" dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{6BB0F30E-FA6E-40B9-88DC-F336A66A15EA}" name="LOB/Project" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{7EEF8C9E-E28F-4C2F-82B3-CCDBBE2BAE5B}" name="Technology Stack" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{C76712CA-C3D0-400A-A5B0-1590E99A3801}" name="Framework" dataDxfId="2"/>
+    <tableColumn id="7" xr3:uid="{D40351DA-4625-4AED-92C1-8C733CE6AAF1}" name="Runtime" dataDxfId="1"/>
+    <tableColumn id="11" xr3:uid="{049BCF70-240C-47F6-81A7-D6DCBBA621E4}" name="Shared Library" dataDxfId="0"/>
     <tableColumn id="10" xr3:uid="{B0EAF2DB-B0F5-4CBD-93BD-4CE41A39352C}" name="Issue"/>
     <tableColumn id="8" xr3:uid="{5C9D9247-EEBA-4739-BB7F-3D0FC59E85E4}" name="Repo Type"/>
   </tableColumns>
@@ -3338,12 +3294,12 @@
   <cols>
     <col min="1" max="1" width="37" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="68.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.5703125" style="9" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17" style="9" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26" style="9" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16" style="9" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.42578125" style="9" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.42578125" style="9" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5703125" style="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17" style="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26" style="8" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16" style="8" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" style="8" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.42578125" style="8" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="80" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="24.28515625" customWidth="1"/>
   </cols>
@@ -3355,22 +3311,22 @@
       <c r="B1" t="s">
         <v>75</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="E1" s="8" t="s">
         <v>122</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="F1" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="G1" s="8" t="s">
         <v>103</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="H1" s="8" t="s">
         <v>111</v>
       </c>
       <c r="I1" t="s">
@@ -3380,1884 +3336,1884 @@
         <v>117</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:10" hidden="1">
       <c r="A2" s="6" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="C2" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E2" s="9" t="s">
+      <c r="D2" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E2" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="F2" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="G2" s="9" t="s">
+      <c r="G2" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="H2" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10">
+      <c r="H2" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" hidden="1">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="C3" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D3" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E3" s="9" t="s">
+      <c r="D3" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E3" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="F3" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="G3" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="H3" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10">
+      <c r="H3" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" hidden="1">
       <c r="A4" s="6" t="s">
         <v>9</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E4" s="9" t="s">
+      <c r="D4" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E4" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="F4" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="G4" s="9" t="s">
+      <c r="G4" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="H4" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10">
+      <c r="H4" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" hidden="1">
       <c r="A5" s="6" t="s">
         <v>11</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E5" s="9" t="s">
+      <c r="D5" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E5" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="F5" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="G5" s="9" t="s">
+      <c r="G5" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="H5" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10">
+      <c r="H5" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" hidden="1">
       <c r="A6" s="6" t="s">
         <v>14</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C6" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E6" s="9" t="s">
+      <c r="D6" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E6" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="F6" s="9" t="s">
+      <c r="F6" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="G6" s="9" t="s">
+      <c r="G6" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="H6" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10">
+      <c r="H6" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" hidden="1">
       <c r="A7" s="6" t="s">
         <v>3</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D7" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E7" s="9" t="s">
+      <c r="D7" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E7" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="F7" s="9" t="s">
+      <c r="F7" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="G7" s="9" t="s">
+      <c r="G7" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="H7" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10">
+      <c r="H7" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" hidden="1">
       <c r="A8" s="6" t="s">
         <v>6</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D8" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E8" s="9" t="s">
+      <c r="D8" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E8" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="F8" s="9" t="s">
+      <c r="F8" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="G8" s="9" t="s">
+      <c r="G8" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="H8" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10">
+      <c r="H8" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" hidden="1">
       <c r="A9" s="6" t="s">
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C9" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D9" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E9" s="9" t="s">
+      <c r="D9" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E9" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="F9" s="9" t="s">
+      <c r="F9" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="G9" s="9" t="s">
+      <c r="G9" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="H9" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10">
+      <c r="H9" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" hidden="1">
       <c r="A10" s="6" t="s">
         <v>12</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="C10" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D10" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E10" s="9" t="s">
+      <c r="D10" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E10" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="F10" s="9" t="s">
+      <c r="F10" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="G10" s="9" t="s">
+      <c r="G10" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="H10" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10">
+      <c r="H10" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" hidden="1">
       <c r="A11" s="6" t="s">
         <v>16</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="C11" s="9" t="s">
+      <c r="C11" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D11" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E11" s="9" t="s">
+      <c r="D11" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E11" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="F11" s="9" t="s">
+      <c r="F11" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="G11" s="9" t="s">
+      <c r="G11" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="H11" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10">
+      <c r="H11" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" hidden="1">
       <c r="A12" s="6" t="s">
         <v>17</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="C12" s="9" t="s">
+      <c r="C12" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D12" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E12" s="9" t="s">
+      <c r="D12" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E12" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="F12" s="9" t="s">
+      <c r="F12" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="G12" s="9" t="s">
+      <c r="G12" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="H12" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10">
+      <c r="H12" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" hidden="1">
       <c r="A13" s="6" t="s">
         <v>19</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="C13" s="9" t="s">
+      <c r="C13" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D13" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E13" s="9" t="s">
+      <c r="D13" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E13" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="F13" s="9" t="s">
+      <c r="F13" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="G13" s="9" t="s">
+      <c r="G13" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="H13" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10">
+      <c r="H13" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" hidden="1">
       <c r="A14" s="6" t="s">
         <v>20</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="C14" s="9" t="s">
+      <c r="C14" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D14" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E14" s="9" t="s">
+      <c r="D14" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E14" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="F14" s="9" t="s">
+      <c r="F14" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="G14" s="9" t="s">
+      <c r="G14" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="H14" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10">
+      <c r="H14" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" hidden="1">
       <c r="A15" s="6" t="s">
         <v>5</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="C15" s="9" t="s">
+      <c r="C15" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D15" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E15" s="9" t="s">
+      <c r="D15" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E15" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="F15" s="9" t="s">
+      <c r="F15" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="G15" s="9" t="s">
+      <c r="G15" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="H15" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10">
+      <c r="H15" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" hidden="1">
       <c r="A16" s="6" t="s">
         <v>18</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="C16" s="9" t="s">
+      <c r="C16" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="D16" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E16" s="9" t="s">
+      <c r="D16" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E16" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="F16" s="9" t="s">
+      <c r="F16" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="G16" s="9" t="s">
+      <c r="G16" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="H16" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9">
+      <c r="H16" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" hidden="1">
       <c r="A17" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="C17" s="9" t="s">
+      <c r="C17" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D17" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E17" s="9" t="s">
+      <c r="D17" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E17" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="F17" s="9" t="s">
+      <c r="F17" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="G17" s="9" t="s">
+      <c r="G17" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="H17" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9">
+      <c r="H17" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" hidden="1">
       <c r="A18" s="6" t="s">
         <v>24</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="C18" s="9" t="s">
+      <c r="C18" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D18" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E18" s="9" t="s">
+      <c r="D18" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E18" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="F18" s="9" t="s">
+      <c r="F18" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="G18" s="9" t="s">
+      <c r="G18" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="H18" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9">
+      <c r="H18" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" hidden="1">
       <c r="A19" s="6" t="s">
         <v>57</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="C19" s="9" t="s">
+      <c r="C19" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D19" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E19" s="9" t="s">
+      <c r="D19" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E19" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="F19" s="9" t="s">
+      <c r="F19" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="G19" s="9" t="s">
+      <c r="G19" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="H19" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9">
+      <c r="H19" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" hidden="1">
       <c r="A20" s="6" t="s">
         <v>53</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="C20" s="9" t="s">
+      <c r="C20" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D20" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E20" s="9" t="s">
+      <c r="D20" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E20" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="F20" s="9" t="s">
+      <c r="F20" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="G20" s="9" t="s">
+      <c r="G20" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="H20" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9">
+      <c r="H20" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" hidden="1">
       <c r="A21" s="6" t="s">
         <v>68</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="C21" s="9" t="s">
+      <c r="C21" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D21" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E21" s="9" t="s">
+      <c r="D21" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E21" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="F21" s="9" t="s">
+      <c r="F21" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="G21" s="9" t="s">
+      <c r="G21" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="H21" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9">
+      <c r="H21" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" hidden="1">
       <c r="A22" s="7" t="s">
         <v>7</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="C22" s="9" t="s">
+      <c r="C22" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="D22" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E22" s="9" t="s">
+      <c r="D22" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E22" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="F22" s="9" t="s">
+      <c r="F22" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="G22" s="9" t="s">
+      <c r="G22" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="I22" s="10" t="s">
+      <c r="I22" s="9" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="23" spans="1:9">
+    <row r="23" spans="1:9" hidden="1">
       <c r="A23" s="7" t="s">
         <v>10</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="C23" s="9" t="s">
+      <c r="C23" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="D23" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E23" s="9" t="s">
+      <c r="D23" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E23" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="F23" s="9" t="s">
+      <c r="F23" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="G23" s="9" t="s">
+      <c r="G23" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="I23" s="10" t="s">
+      <c r="I23" s="9" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="24" spans="1:9">
+    <row r="24" spans="1:9" hidden="1">
       <c r="A24" s="7" t="s">
         <v>13</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="C24" s="9" t="s">
+      <c r="C24" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="D24" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E24" s="9" t="s">
+      <c r="D24" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E24" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="F24" s="9" t="s">
+      <c r="F24" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="G24" s="9" t="s">
+      <c r="G24" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="I24" s="10" t="s">
+      <c r="I24" s="9" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="25" spans="1:9" hidden="1">
-      <c r="A25" s="8" t="s">
+    <row r="25" spans="1:9">
+      <c r="A25" s="6" t="s">
         <v>0</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="C25" s="9" t="s">
+      <c r="C25" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D25" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E25" s="9" t="s">
+      <c r="D25" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E25" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="F25" s="9" t="s">
+      <c r="F25" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="G25" s="9" t="s">
+      <c r="G25" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H25" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" hidden="1">
-      <c r="A26" s="8" t="s">
+      <c r="H25" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9">
+      <c r="A26" s="6" t="s">
         <v>21</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="C26" s="9" t="s">
+      <c r="C26" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="D26" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E26" s="9" t="s">
+      <c r="D26" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E26" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="F26" s="9" t="s">
+      <c r="F26" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="G26" s="9" t="s">
+      <c r="G26" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H26" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" hidden="1">
-      <c r="A27" s="8" t="s">
+      <c r="H26" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9">
+      <c r="A27" s="6" t="s">
         <v>22</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="C27" s="9" t="s">
+      <c r="C27" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="D27" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E27" s="9" t="s">
+      <c r="D27" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E27" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="F27" s="9" t="s">
+      <c r="F27" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="G27" s="9" t="s">
+      <c r="G27" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H27" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" hidden="1">
-      <c r="A28" s="8" t="s">
+      <c r="H27" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9">
+      <c r="A28" s="6" t="s">
         <v>23</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C28" s="9" t="s">
+      <c r="C28" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D28" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E28" s="9" t="s">
+      <c r="D28" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E28" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="F28" s="9" t="s">
+      <c r="F28" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="G28" s="9" t="s">
+      <c r="G28" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H28" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" hidden="1">
-      <c r="A29" s="8" t="s">
+      <c r="H28" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9">
+      <c r="A29" s="6" t="s">
         <v>25</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C29" s="9" t="s">
+      <c r="C29" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D29" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E29" s="9" t="s">
+      <c r="D29" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E29" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="F29" s="9" t="s">
+      <c r="F29" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="G29" s="9" t="s">
+      <c r="G29" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H29" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" hidden="1">
-      <c r="A30" s="8" t="s">
+      <c r="H29" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9">
+      <c r="A30" s="11" t="s">
         <v>26</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="C30" s="9" t="s">
+      <c r="C30" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="D30" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E30" s="9" t="s">
+      <c r="D30" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E30" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="G30" s="9" t="s">
+      <c r="G30" s="8" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="31" spans="1:9" hidden="1">
-      <c r="A31" s="8" t="s">
+    <row r="31" spans="1:9">
+      <c r="A31" s="6" t="s">
         <v>27</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="C31" s="9" t="s">
+      <c r="C31" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="D31" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E31" s="9" t="s">
+      <c r="D31" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E31" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="F31" s="9" t="s">
+      <c r="F31" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="G31" s="9" t="s">
+      <c r="G31" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H31" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" hidden="1">
-      <c r="A32" s="8" t="s">
+      <c r="H31" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9">
+      <c r="A32" s="6" t="s">
         <v>28</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="C32" s="9" t="s">
+      <c r="C32" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="D32" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E32" s="9" t="s">
+      <c r="D32" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E32" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="F32" s="9" t="s">
+      <c r="F32" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="G32" s="9" t="s">
+      <c r="G32" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H32" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" hidden="1">
-      <c r="A33" s="8" t="s">
+      <c r="H32" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10">
+      <c r="A33" s="6" t="s">
         <v>29</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="C33" s="9" t="s">
+      <c r="C33" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="D33" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E33" s="9" t="s">
+      <c r="D33" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E33" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="F33" s="9" t="s">
+      <c r="F33" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="G33" s="9" t="s">
+      <c r="G33" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H33" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10" hidden="1">
-      <c r="A34" s="8" t="s">
+      <c r="H33" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10">
+      <c r="A34" s="6" t="s">
         <v>30</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C34" s="9" t="s">
+      <c r="C34" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D34" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E34" s="9" t="s">
+      <c r="D34" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E34" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="F34" s="9" t="s">
+      <c r="F34" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="G34" s="9" t="s">
+      <c r="G34" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H34" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10" hidden="1">
-      <c r="A35" s="8" t="s">
+      <c r="H34" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10">
+      <c r="A35" s="6" t="s">
         <v>31</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="C35" s="9" t="s">
+      <c r="C35" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="D35" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E35" s="9" t="s">
+      <c r="D35" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E35" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="G35" s="9" t="s">
+      <c r="G35" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H35" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="I35" s="11"/>
-    </row>
-    <row r="36" spans="1:10" hidden="1">
-      <c r="A36" s="8" t="s">
+      <c r="H35" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="I35" s="10"/>
+    </row>
+    <row r="36" spans="1:10">
+      <c r="A36" s="11" t="s">
         <v>32</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="C36" s="9" t="s">
+      <c r="C36" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D36" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E36" s="9" t="s">
+      <c r="D36" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E36" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="G36" s="9" t="s">
+      <c r="G36" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H36" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" hidden="1">
-      <c r="A37" s="8" t="s">
+      <c r="H36" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10">
+      <c r="A37" s="6" t="s">
         <v>34</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="C37" s="9" t="s">
+      <c r="C37" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="D37" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E37" s="9" t="s">
+      <c r="D37" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E37" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="F37" s="9" t="s">
+      <c r="F37" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="G37" s="9" t="s">
+      <c r="G37" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H37" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10" hidden="1">
-      <c r="A38" s="8" t="s">
+      <c r="H37" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10">
+      <c r="A38" s="6" t="s">
         <v>35</v>
       </c>
       <c r="B38" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="C38" s="9" t="s">
+      <c r="C38" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="D38" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E38" s="9" t="s">
+      <c r="D38" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E38" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="F38" s="9" t="s">
+      <c r="F38" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="G38" s="9" t="s">
+      <c r="G38" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H38" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10" hidden="1">
-      <c r="A39" s="8" t="s">
+      <c r="H38" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10">
+      <c r="A39" s="11" t="s">
         <v>36</v>
       </c>
       <c r="B39" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="C39" s="9" t="s">
+      <c r="C39" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D39" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E39" s="9" t="s">
+      <c r="D39" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E39" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="G39" s="9" t="s">
+      <c r="G39" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H39" s="9" t="s">
+      <c r="H39" s="8" t="s">
         <v>115</v>
       </c>
       <c r="J39" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="40" spans="1:10" hidden="1">
-      <c r="A40" s="8" t="s">
+    <row r="40" spans="1:10">
+      <c r="A40" s="6" t="s">
         <v>37</v>
       </c>
       <c r="B40" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C40" s="9" t="s">
+      <c r="C40" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D40" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E40" s="9" t="s">
+      <c r="D40" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E40" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="F40" s="9" t="s">
+      <c r="F40" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="G40" s="9" t="s">
+      <c r="G40" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H40" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="41" spans="1:10" hidden="1">
-      <c r="A41" s="8" t="s">
+      <c r="H40" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10">
+      <c r="A41" s="6" t="s">
         <v>38</v>
       </c>
       <c r="B41" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C41" s="9" t="s">
+      <c r="C41" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D41" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E41" s="9" t="s">
+      <c r="D41" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E41" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="F41" s="9" t="s">
+      <c r="F41" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="G41" s="9" t="s">
+      <c r="G41" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H41" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="42" spans="1:10" hidden="1">
-      <c r="A42" s="8" t="s">
+      <c r="H41" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10">
+      <c r="A42" s="6" t="s">
         <v>39</v>
       </c>
       <c r="B42" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C42" s="9" t="s">
+      <c r="C42" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D42" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E42" s="9" t="s">
+      <c r="D42" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E42" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="F42" s="9" t="s">
+      <c r="F42" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="G42" s="9" t="s">
+      <c r="G42" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H42" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="43" spans="1:10" hidden="1">
-      <c r="A43" s="8" t="s">
+      <c r="H42" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10">
+      <c r="A43" s="6" t="s">
         <v>40</v>
       </c>
       <c r="B43" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="C43" s="9" t="s">
+      <c r="C43" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D43" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E43" s="9" t="s">
+      <c r="D43" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E43" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="G43" s="9" t="s">
+      <c r="G43" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H43" s="9" t="s">
+      <c r="H43" s="8" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="44" spans="1:10" hidden="1">
-      <c r="A44" s="8" t="s">
+    <row r="44" spans="1:10">
+      <c r="A44" s="6" t="s">
         <v>41</v>
       </c>
       <c r="B44" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="C44" s="9" t="s">
+      <c r="C44" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D44" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E44" s="9" t="s">
+      <c r="D44" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E44" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="G44" s="9" t="s">
+      <c r="G44" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H44" s="9" t="s">
+      <c r="H44" s="8" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="45" spans="1:10" hidden="1">
-      <c r="A45" s="8" t="s">
+    <row r="45" spans="1:10">
+      <c r="A45" s="6" t="s">
         <v>43</v>
       </c>
       <c r="B45" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="C45" s="9" t="s">
+      <c r="C45" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D45" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E45" s="9" t="s">
+      <c r="D45" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E45" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="G45" s="9" t="s">
+      <c r="G45" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H45" s="9" t="s">
+      <c r="H45" s="8" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="46" spans="1:10" hidden="1">
-      <c r="A46" s="8" t="s">
+    <row r="46" spans="1:10">
+      <c r="A46" s="6" t="s">
         <v>44</v>
       </c>
       <c r="B46" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C46" s="9" t="s">
+      <c r="C46" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D46" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E46" s="9" t="s">
+      <c r="D46" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E46" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="F46" s="9" t="s">
+      <c r="F46" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="G46" s="9" t="s">
+      <c r="G46" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H46" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="47" spans="1:10" hidden="1">
-      <c r="A47" s="8" t="s">
+      <c r="H46" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10">
+      <c r="A47" s="6" t="s">
         <v>45</v>
       </c>
       <c r="B47" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C47" s="9" t="s">
+      <c r="C47" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D47" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E47" s="9" t="s">
+      <c r="D47" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E47" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="F47" s="9" t="s">
+      <c r="F47" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="G47" s="9" t="s">
+      <c r="G47" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H47" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="48" spans="1:10" hidden="1">
-      <c r="A48" s="8" t="s">
+      <c r="H47" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10">
+      <c r="A48" s="6" t="s">
         <v>46</v>
       </c>
       <c r="B48" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C48" s="9" t="s">
+      <c r="C48" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D48" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E48" s="9" t="s">
+      <c r="D48" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E48" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="F48" s="9" t="s">
+      <c r="F48" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="G48" s="9" t="s">
+      <c r="G48" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H48" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="49" spans="1:10" hidden="1">
-      <c r="A49" s="8" t="s">
+      <c r="H48" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10">
+      <c r="A49" s="6" t="s">
         <v>47</v>
       </c>
       <c r="B49" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C49" s="9" t="s">
+      <c r="C49" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D49" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E49" s="9" t="s">
+      <c r="D49" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E49" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="F49" s="9" t="s">
+      <c r="F49" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="G49" s="9" t="s">
+      <c r="G49" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H49" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="50" spans="1:10" hidden="1">
-      <c r="A50" s="8" t="s">
+      <c r="H49" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10">
+      <c r="A50" s="6" t="s">
         <v>48</v>
       </c>
       <c r="B50" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C50" s="9" t="s">
+      <c r="C50" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D50" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E50" s="9" t="s">
+      <c r="D50" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E50" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="F50" s="9" t="s">
+      <c r="F50" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="G50" s="9" t="s">
+      <c r="G50" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H50" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="51" spans="1:10" hidden="1">
-      <c r="A51" s="8" t="s">
+      <c r="H50" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10">
+      <c r="A51" s="6" t="s">
         <v>49</v>
       </c>
       <c r="B51" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C51" s="9" t="s">
+      <c r="C51" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D51" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E51" s="9" t="s">
+      <c r="D51" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E51" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="F51" s="9" t="s">
+      <c r="F51" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="G51" s="9" t="s">
+      <c r="G51" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H51" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="52" spans="1:10" hidden="1">
-      <c r="A52" s="8" t="s">
+      <c r="H51" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10">
+      <c r="A52" s="6" t="s">
         <v>50</v>
       </c>
       <c r="B52" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C52" s="9" t="s">
+      <c r="C52" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D52" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E52" s="9" t="s">
+      <c r="D52" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E52" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="F52" s="9" t="s">
+      <c r="F52" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="G52" s="9" t="s">
+      <c r="G52" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H52" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="53" spans="1:10" hidden="1">
-      <c r="A53" s="8" t="s">
+      <c r="H52" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10">
+      <c r="A53" s="6" t="s">
         <v>51</v>
       </c>
       <c r="B53" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C53" s="9" t="s">
+      <c r="C53" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D53" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E53" s="9" t="s">
+      <c r="D53" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E53" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="F53" s="9" t="s">
+      <c r="F53" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="G53" s="9" t="s">
+      <c r="G53" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H53" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="54" spans="1:10" hidden="1">
-      <c r="A54" s="8" t="s">
+      <c r="H53" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10">
+      <c r="A54" s="6" t="s">
         <v>52</v>
       </c>
       <c r="B54" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C54" s="9" t="s">
+      <c r="C54" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D54" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E54" s="9" t="s">
+      <c r="D54" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E54" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="F54" s="9" t="s">
+      <c r="F54" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="G54" s="9" t="s">
+      <c r="G54" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H54" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="55" spans="1:10" hidden="1">
-      <c r="A55" s="8" t="s">
+      <c r="H54" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10">
+      <c r="A55" s="6" t="s">
         <v>54</v>
       </c>
       <c r="B55" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C55" s="9" t="s">
+      <c r="C55" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D55" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E55" s="9" t="s">
+      <c r="D55" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E55" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="F55" s="9" t="s">
+      <c r="F55" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="G55" s="9" t="s">
+      <c r="G55" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H55" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="56" spans="1:10" hidden="1">
-      <c r="A56" s="8" t="s">
+      <c r="H55" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10">
+      <c r="A56" s="6" t="s">
         <v>55</v>
       </c>
       <c r="B56" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C56" s="9" t="s">
+      <c r="C56" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D56" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E56" s="9" t="s">
+      <c r="D56" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E56" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="F56" s="9" t="s">
+      <c r="F56" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="G56" s="9" t="s">
+      <c r="G56" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H56" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="57" spans="1:10" hidden="1">
-      <c r="A57" s="8" t="s">
+      <c r="H56" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10">
+      <c r="A57" s="6" t="s">
         <v>56</v>
       </c>
       <c r="B57" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C57" s="9" t="s">
+      <c r="C57" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D57" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E57" s="9" t="s">
+      <c r="D57" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E57" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="F57" s="9" t="s">
+      <c r="F57" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="G57" s="9" t="s">
+      <c r="G57" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H57" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="58" spans="1:10" hidden="1">
-      <c r="A58" s="8" t="s">
+      <c r="H57" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10">
+      <c r="A58" s="6" t="s">
         <v>58</v>
       </c>
       <c r="B58" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C58" s="9" t="s">
+      <c r="C58" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D58" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E58" s="9" t="s">
+      <c r="D58" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E58" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="F58" s="9" t="s">
+      <c r="F58" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="G58" s="9" t="s">
+      <c r="G58" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H58" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="59" spans="1:10" hidden="1">
-      <c r="A59" s="8" t="s">
+      <c r="H58" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10">
+      <c r="A59" s="6" t="s">
         <v>59</v>
       </c>
       <c r="B59" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C59" s="9" t="s">
+      <c r="C59" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D59" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E59" s="9" t="s">
+      <c r="D59" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E59" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="F59" s="9" t="s">
+      <c r="F59" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="G59" s="9" t="s">
+      <c r="G59" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H59" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="60" spans="1:10" hidden="1">
-      <c r="A60" s="8" t="s">
+      <c r="H59" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10">
+      <c r="A60" s="6" t="s">
         <v>60</v>
       </c>
       <c r="B60" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C60" s="9" t="s">
+      <c r="C60" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D60" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E60" s="9" t="s">
+      <c r="D60" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E60" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="F60" s="9" t="s">
+      <c r="F60" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="G60" s="9" t="s">
+      <c r="G60" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H60" s="9" t="s">
+      <c r="H60" s="8" t="s">
         <v>115</v>
       </c>
       <c r="J60" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="61" spans="1:10" hidden="1">
-      <c r="A61" s="8" t="s">
+    <row r="61" spans="1:10">
+      <c r="A61" s="6" t="s">
         <v>61</v>
       </c>
       <c r="B61" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C61" s="9" t="s">
+      <c r="C61" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D61" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E61" s="9" t="s">
+      <c r="D61" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E61" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="F61" s="9" t="s">
+      <c r="F61" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="G61" s="9" t="s">
+      <c r="G61" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H61" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="62" spans="1:10" hidden="1">
-      <c r="A62" s="8" t="s">
+      <c r="H61" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10">
+      <c r="A62" s="6" t="s">
         <v>62</v>
       </c>
       <c r="B62" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C62" s="9" t="s">
+      <c r="C62" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D62" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E62" s="9" t="s">
+      <c r="D62" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E62" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="F62" s="9" t="s">
+      <c r="F62" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="G62" s="9" t="s">
+      <c r="G62" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H62" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="63" spans="1:10" hidden="1">
-      <c r="A63" s="8" t="s">
+      <c r="H62" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10">
+      <c r="A63" s="6" t="s">
         <v>64</v>
       </c>
       <c r="B63" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C63" s="9" t="s">
+      <c r="C63" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D63" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E63" s="9" t="s">
+      <c r="D63" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E63" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="F63" s="9" t="s">
+      <c r="F63" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="G63" s="9" t="s">
+      <c r="G63" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H63" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="64" spans="1:10" hidden="1">
-      <c r="A64" s="8" t="s">
+      <c r="H63" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10">
+      <c r="A64" s="6" t="s">
         <v>65</v>
       </c>
       <c r="B64" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C64" s="9" t="s">
+      <c r="C64" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D64" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E64" s="9" t="s">
+      <c r="D64" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E64" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="F64" s="9" t="s">
+      <c r="F64" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="G64" s="9" t="s">
+      <c r="G64" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H64" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="65" spans="1:9" hidden="1">
-      <c r="A65" s="8" t="s">
+      <c r="H64" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9">
+      <c r="A65" s="6" t="s">
         <v>66</v>
       </c>
       <c r="B65" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C65" s="9" t="s">
+      <c r="C65" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D65" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E65" s="9" t="s">
+      <c r="D65" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E65" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="F65" s="9" t="s">
+      <c r="F65" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="G65" s="9" t="s">
+      <c r="G65" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H65" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="66" spans="1:9" hidden="1">
-      <c r="A66" s="8" t="s">
+      <c r="H65" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9">
+      <c r="A66" s="6" t="s">
         <v>67</v>
       </c>
       <c r="B66" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C66" s="9" t="s">
+      <c r="C66" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D66" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E66" s="9" t="s">
+      <c r="D66" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E66" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="F66" s="9" t="s">
+      <c r="F66" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="G66" s="9" t="s">
+      <c r="G66" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H66" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="67" spans="1:9" hidden="1">
-      <c r="A67" s="8" t="s">
+      <c r="H66" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9">
+      <c r="A67" s="6" t="s">
         <v>69</v>
       </c>
       <c r="B67" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C67" s="9" t="s">
+      <c r="C67" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D67" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E67" s="9" t="s">
+      <c r="D67" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E67" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="F67" s="9" t="s">
+      <c r="F67" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="G67" s="9" t="s">
+      <c r="G67" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H67" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="68" spans="1:9" hidden="1">
-      <c r="A68" s="8" t="s">
+      <c r="H67" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9">
+      <c r="A68" s="6" t="s">
         <v>70</v>
       </c>
       <c r="B68" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C68" s="9" t="s">
+      <c r="C68" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D68" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E68" s="9" t="s">
+      <c r="D68" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E68" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="F68" s="9" t="s">
+      <c r="F68" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="G68" s="9" t="s">
+      <c r="G68" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H68" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="69" spans="1:9" hidden="1">
-      <c r="A69" s="8" t="s">
+      <c r="H68" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9">
+      <c r="A69" s="6" t="s">
         <v>71</v>
       </c>
       <c r="B69" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C69" s="9" t="s">
+      <c r="C69" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D69" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E69" s="9" t="s">
+      <c r="D69" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E69" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="F69" s="9" t="s">
+      <c r="F69" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="G69" s="9" t="s">
+      <c r="G69" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H69" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="70" spans="1:9" hidden="1">
-      <c r="A70" s="8" t="s">
+      <c r="H69" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9">
+      <c r="A70" s="6" t="s">
         <v>72</v>
       </c>
       <c r="B70" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C70" s="9" t="s">
+      <c r="C70" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D70" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E70" s="9" t="s">
+      <c r="D70" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E70" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="F70" s="9" t="s">
+      <c r="F70" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="G70" s="9" t="s">
+      <c r="G70" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H70" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="71" spans="1:9" hidden="1">
+      <c r="H70" s="8" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="71" spans="1:9">
       <c r="A71" s="7" t="s">
         <v>33</v>
       </c>
       <c r="B71" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="C71" s="9" t="s">
+      <c r="C71" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="D71" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E71" s="9" t="s">
+      <c r="D71" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E71" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="G71" s="9" t="s">
+      <c r="G71" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="I71" s="10" t="s">
+      <c r="I71" s="9" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="72" spans="1:9" hidden="1">
-      <c r="A72" s="12" t="s">
+    <row r="72" spans="1:9">
+      <c r="A72" s="7" t="s">
         <v>42</v>
       </c>
       <c r="B72" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="C72" s="9" t="s">
+      <c r="C72" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D72" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E72" s="9" t="s">
+      <c r="D72" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E72" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="G72" s="9" t="s">
+      <c r="G72" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H72" s="9" t="s">
+      <c r="H72" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="I72" s="10" t="s">
+      <c r="I72" s="9" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="73" spans="1:9" hidden="1">
-      <c r="A73" s="12" t="s">
+    <row r="73" spans="1:9">
+      <c r="A73" s="7" t="s">
         <v>63</v>
       </c>
       <c r="B73" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="C73" s="9" t="s">
+      <c r="C73" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="D73" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E73" s="9" t="s">
+      <c r="D73" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E73" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="G73" s="9" t="s">
+      <c r="G73" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H73" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="I73" s="10" t="s">
+      <c r="H73" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="I73" s="9" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="74" spans="1:9" hidden="1">
-      <c r="A74" s="12" t="s">
+    <row r="74" spans="1:9">
+      <c r="A74" s="7" t="s">
         <v>73</v>
       </c>
       <c r="B74" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C74" s="9" t="s">
+      <c r="C74" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D74" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E74" s="9" t="s">
+      <c r="D74" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E74" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="F74" s="9" t="s">
+      <c r="F74" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="G74" s="9" t="s">
+      <c r="G74" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H74" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="I74" s="10" t="s">
+      <c r="H74" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="I74" s="9" t="s">
         <v>110</v>
       </c>
     </row>

</xml_diff>